<commit_message>
Separate trip travel from daily itinerary
</commit_message>
<xml_diff>
--- a/outputs/01a0775c-925e-7713-9822-42450cb2f4b6/Hope-Sojourns-Trip-Bulk-Import-Template.xlsx
+++ b/outputs/01a0775c-925e-7713-9822-42450cb2f4b6/Hope-Sojourns-Trip-Bulk-Import-Template.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R59db7b4751bb48b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R53a25dc4a7b74481"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ministries" sheetId="3" r:id="R9c24e96e6b604bdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team" sheetId="4" r:id="R3369965932114a18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Partners" sheetId="5" r:id="Rffc2827c1f4340e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="6" r:id="R66a71fa3cde74b15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accounts" sheetId="7" r:id="R6e9750fa9815400e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="8" r:id="Rf6dd2bc808fc432f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Allocations" sheetId="9" r:id="R5b701354c3794b3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charges" sheetId="10" r:id="R7e169865e0cb4888"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support" sheetId="11" r:id="Re54d9ce3368f44ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments" sheetId="12" r:id="R9c5ebf93349e47bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invites" sheetId="13" r:id="Rfea516d75d904692"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rfaab6a5b1f01430e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="R9371f455f5be408d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ministries" sheetId="3" r:id="Re911094b5c414368"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team" sheetId="4" r:id="R04d49d7d73ae4ac8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Partners" sheetId="5" r:id="R2cec68d214fd4f39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="6" r:id="R56c00128f5a54b62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accounts" sheetId="7" r:id="Rf30de2b8996148f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="8" r:id="R7dad3664eab2497d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Allocations" sheetId="9" r:id="R0f342ae717084d25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charges" sheetId="10" r:id="R003eaa29db624002"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support" sheetId="11" r:id="R1dbfc540c02f44ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments" sheetId="12" r:id="Rfb837cc1fe554bce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invites" sheetId="13" r:id="R41d28701bfc84f82"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -397,9 +397,9 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="HsContentImport" displayName="HsContentImport" ref="A4:N104" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N104"/>
-  <x:tableColumns count="14">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="HsContentImport" displayName="HsContentImport" ref="A4:S104" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:S104"/>
+  <x:tableColumns count="19">
     <x:tableColumn id="1" name="Import Ref"/>
     <x:tableColumn id="2" name="Content Type"/>
     <x:tableColumn id="3" name="Title"/>
@@ -411,9 +411,14 @@
     <x:tableColumn id="9" name="Visibility"/>
     <x:tableColumn id="10" name="Publication Status"/>
     <x:tableColumn id="11" name="Sort Order"/>
-    <x:tableColumn id="12" name="Record ID"/>
-    <x:tableColumn id="13" name="Original Updated At"/>
-    <x:tableColumn id="14" name="Original Fingerprint"/>
+    <x:tableColumn id="12" name="Arrival Date"/>
+    <x:tableColumn id="13" name="Arrival Time"/>
+    <x:tableColumn id="14" name="Arrival Location"/>
+    <x:tableColumn id="15" name="Travel Mode"/>
+    <x:tableColumn id="16" name="Service Number"/>
+    <x:tableColumn id="17" name="Record ID"/>
+    <x:tableColumn id="18" name="Original Updated At"/>
+    <x:tableColumn id="19" name="Original Fingerprint"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -2395,7 +2400,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54fbee42fcdc4a6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R349788d5a688424e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3816,7 +3821,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43777fdbb2c34600"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9359501715f448a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6206,7 +6211,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3777480f84542d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc383aca10fe5433f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7298,7 +7303,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3eb80480e8c412e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c4962b71f504ce7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9896,7 +9901,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64a62e0cedb54fa5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5845eb3c8cf843f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11956,7 +11961,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7b143d395bf406d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re20296bcdfba41fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13493,7 +13498,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15bd3f05cf5b4f5d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9f14c656e614c7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14585,7 +14590,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a8c13ce999c4e4a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2dca55a2e5544cf6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14610,7 +14615,12 @@
     <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="20" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="18" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -14630,10 +14640,15 @@
       <x:c r="L1" s="20"/>
       <x:c r="M1" s="20"/>
       <x:c r="N1" s="20"/>
+      <x:c r="O1" s="20"/>
+      <x:c r="P1" s="20"/>
+      <x:c r="Q1" s="20"/>
+      <x:c r="R1" s="20"/>
+      <x:c r="S1" s="20"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="24" t="str">
-        <x:v>Load itinerary entries, devotionals, instructions, resources, updates, and overview content.</x:v>
+        <x:v>Use travel for transport legs and itinerary for daily activities. Travel Event Date, Event Time, and Location describe departure; use local times and travelers or admin visibility.</x:v>
       </x:c>
       <x:c r="B2" s="24"/>
       <x:c r="C2" s="24"/>
@@ -14648,6 +14663,11 @@
       <x:c r="L2" s="24"/>
       <x:c r="M2" s="24"/>
       <x:c r="N2" s="24"/>
+      <x:c r="O2" s="24"/>
+      <x:c r="P2" s="24"/>
+      <x:c r="Q2" s="24"/>
+      <x:c r="R2" s="24"/>
+      <x:c r="S2" s="24"/>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="28" t="str">
@@ -14666,6 +14686,11 @@
       <x:c r="L3" s="28"/>
       <x:c r="M3" s="28"/>
       <x:c r="N3" s="28"/>
+      <x:c r="O3" s="28"/>
+      <x:c r="P3" s="28"/>
+      <x:c r="Q3" s="28"/>
+      <x:c r="R3" s="28"/>
+      <x:c r="S3" s="28"/>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="33" t="str">
@@ -14702,12 +14727,27 @@
         <x:v>Sort Order</x:v>
       </x:c>
       <x:c r="L4" s="33" t="str">
+        <x:v>Arrival Date</x:v>
+      </x:c>
+      <x:c r="M4" s="33" t="str">
+        <x:v>Arrival Time</x:v>
+      </x:c>
+      <x:c r="N4" s="33" t="str">
+        <x:v>Arrival Location</x:v>
+      </x:c>
+      <x:c r="O4" s="33" t="str">
+        <x:v>Travel Mode</x:v>
+      </x:c>
+      <x:c r="P4" s="33" t="str">
+        <x:v>Service Number</x:v>
+      </x:c>
+      <x:c r="Q4" s="33" t="str">
         <x:v>Record ID</x:v>
       </x:c>
-      <x:c r="M4" s="33" t="str">
+      <x:c r="R4" s="33" t="str">
         <x:v>Original Updated At</x:v>
       </x:c>
-      <x:c r="N4" s="33" t="str">
+      <x:c r="S4" s="33" t="str">
         <x:v>Original Fingerprint</x:v>
       </x:c>
     </x:row>
@@ -14723,9 +14763,14 @@
       <x:c r="I5" s="37"/>
       <x:c r="J5" s="37"/>
       <x:c r="K5" s="40"/>
-      <x:c r="L5" s="38"/>
-      <x:c r="M5" s="38"/>
-      <x:c r="N5" s="38"/>
+      <x:c r="L5" s="39"/>
+      <x:c r="M5" s="37"/>
+      <x:c r="N5" s="37"/>
+      <x:c r="O5" s="37"/>
+      <x:c r="P5" s="37"/>
+      <x:c r="Q5" s="38"/>
+      <x:c r="R5" s="38"/>
+      <x:c r="S5" s="38"/>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="37"/>
@@ -14739,9 +14784,14 @@
       <x:c r="I6" s="37"/>
       <x:c r="J6" s="37"/>
       <x:c r="K6" s="40"/>
-      <x:c r="L6" s="38"/>
-      <x:c r="M6" s="38"/>
-      <x:c r="N6" s="38"/>
+      <x:c r="L6" s="39"/>
+      <x:c r="M6" s="37"/>
+      <x:c r="N6" s="37"/>
+      <x:c r="O6" s="37"/>
+      <x:c r="P6" s="37"/>
+      <x:c r="Q6" s="38"/>
+      <x:c r="R6" s="38"/>
+      <x:c r="S6" s="38"/>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
       <x:c r="A7" s="37"/>
@@ -14755,9 +14805,14 @@
       <x:c r="I7" s="37"/>
       <x:c r="J7" s="37"/>
       <x:c r="K7" s="40"/>
-      <x:c r="L7" s="38"/>
-      <x:c r="M7" s="38"/>
-      <x:c r="N7" s="38"/>
+      <x:c r="L7" s="39"/>
+      <x:c r="M7" s="37"/>
+      <x:c r="N7" s="37"/>
+      <x:c r="O7" s="37"/>
+      <x:c r="P7" s="37"/>
+      <x:c r="Q7" s="38"/>
+      <x:c r="R7" s="38"/>
+      <x:c r="S7" s="38"/>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="37"/>
@@ -14771,9 +14826,14 @@
       <x:c r="I8" s="37"/>
       <x:c r="J8" s="37"/>
       <x:c r="K8" s="40"/>
-      <x:c r="L8" s="38"/>
-      <x:c r="M8" s="38"/>
-      <x:c r="N8" s="38"/>
+      <x:c r="L8" s="39"/>
+      <x:c r="M8" s="37"/>
+      <x:c r="N8" s="37"/>
+      <x:c r="O8" s="37"/>
+      <x:c r="P8" s="37"/>
+      <x:c r="Q8" s="38"/>
+      <x:c r="R8" s="38"/>
+      <x:c r="S8" s="38"/>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="37"/>
@@ -14787,9 +14847,14 @@
       <x:c r="I9" s="37"/>
       <x:c r="J9" s="37"/>
       <x:c r="K9" s="40"/>
-      <x:c r="L9" s="38"/>
-      <x:c r="M9" s="38"/>
-      <x:c r="N9" s="38"/>
+      <x:c r="L9" s="39"/>
+      <x:c r="M9" s="37"/>
+      <x:c r="N9" s="37"/>
+      <x:c r="O9" s="37"/>
+      <x:c r="P9" s="37"/>
+      <x:c r="Q9" s="38"/>
+      <x:c r="R9" s="38"/>
+      <x:c r="S9" s="38"/>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="37"/>
@@ -14803,9 +14868,14 @@
       <x:c r="I10" s="37"/>
       <x:c r="J10" s="37"/>
       <x:c r="K10" s="40"/>
-      <x:c r="L10" s="38"/>
-      <x:c r="M10" s="38"/>
-      <x:c r="N10" s="38"/>
+      <x:c r="L10" s="39"/>
+      <x:c r="M10" s="37"/>
+      <x:c r="N10" s="37"/>
+      <x:c r="O10" s="37"/>
+      <x:c r="P10" s="37"/>
+      <x:c r="Q10" s="38"/>
+      <x:c r="R10" s="38"/>
+      <x:c r="S10" s="38"/>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="37"/>
@@ -14819,9 +14889,14 @@
       <x:c r="I11" s="37"/>
       <x:c r="J11" s="37"/>
       <x:c r="K11" s="40"/>
-      <x:c r="L11" s="38"/>
-      <x:c r="M11" s="38"/>
-      <x:c r="N11" s="38"/>
+      <x:c r="L11" s="39"/>
+      <x:c r="M11" s="37"/>
+      <x:c r="N11" s="37"/>
+      <x:c r="O11" s="37"/>
+      <x:c r="P11" s="37"/>
+      <x:c r="Q11" s="38"/>
+      <x:c r="R11" s="38"/>
+      <x:c r="S11" s="38"/>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="37"/>
@@ -14835,9 +14910,14 @@
       <x:c r="I12" s="37"/>
       <x:c r="J12" s="37"/>
       <x:c r="K12" s="40"/>
-      <x:c r="L12" s="38"/>
-      <x:c r="M12" s="38"/>
-      <x:c r="N12" s="38"/>
+      <x:c r="L12" s="39"/>
+      <x:c r="M12" s="37"/>
+      <x:c r="N12" s="37"/>
+      <x:c r="O12" s="37"/>
+      <x:c r="P12" s="37"/>
+      <x:c r="Q12" s="38"/>
+      <x:c r="R12" s="38"/>
+      <x:c r="S12" s="38"/>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="37"/>
@@ -14851,9 +14931,14 @@
       <x:c r="I13" s="37"/>
       <x:c r="J13" s="37"/>
       <x:c r="K13" s="40"/>
-      <x:c r="L13" s="38"/>
-      <x:c r="M13" s="38"/>
-      <x:c r="N13" s="38"/>
+      <x:c r="L13" s="39"/>
+      <x:c r="M13" s="37"/>
+      <x:c r="N13" s="37"/>
+      <x:c r="O13" s="37"/>
+      <x:c r="P13" s="37"/>
+      <x:c r="Q13" s="38"/>
+      <x:c r="R13" s="38"/>
+      <x:c r="S13" s="38"/>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="37"/>
@@ -14867,9 +14952,14 @@
       <x:c r="I14" s="37"/>
       <x:c r="J14" s="37"/>
       <x:c r="K14" s="40"/>
-      <x:c r="L14" s="38"/>
-      <x:c r="M14" s="38"/>
-      <x:c r="N14" s="38"/>
+      <x:c r="L14" s="39"/>
+      <x:c r="M14" s="37"/>
+      <x:c r="N14" s="37"/>
+      <x:c r="O14" s="37"/>
+      <x:c r="P14" s="37"/>
+      <x:c r="Q14" s="38"/>
+      <x:c r="R14" s="38"/>
+      <x:c r="S14" s="38"/>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="37"/>
@@ -14883,9 +14973,14 @@
       <x:c r="I15" s="37"/>
       <x:c r="J15" s="37"/>
       <x:c r="K15" s="40"/>
-      <x:c r="L15" s="38"/>
-      <x:c r="M15" s="38"/>
-      <x:c r="N15" s="38"/>
+      <x:c r="L15" s="39"/>
+      <x:c r="M15" s="37"/>
+      <x:c r="N15" s="37"/>
+      <x:c r="O15" s="37"/>
+      <x:c r="P15" s="37"/>
+      <x:c r="Q15" s="38"/>
+      <x:c r="R15" s="38"/>
+      <x:c r="S15" s="38"/>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
       <x:c r="A16" s="37"/>
@@ -14899,9 +14994,14 @@
       <x:c r="I16" s="37"/>
       <x:c r="J16" s="37"/>
       <x:c r="K16" s="40"/>
-      <x:c r="L16" s="38"/>
-      <x:c r="M16" s="38"/>
-      <x:c r="N16" s="38"/>
+      <x:c r="L16" s="39"/>
+      <x:c r="M16" s="37"/>
+      <x:c r="N16" s="37"/>
+      <x:c r="O16" s="37"/>
+      <x:c r="P16" s="37"/>
+      <x:c r="Q16" s="38"/>
+      <x:c r="R16" s="38"/>
+      <x:c r="S16" s="38"/>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="37"/>
@@ -14915,9 +15015,14 @@
       <x:c r="I17" s="37"/>
       <x:c r="J17" s="37"/>
       <x:c r="K17" s="40"/>
-      <x:c r="L17" s="38"/>
-      <x:c r="M17" s="38"/>
-      <x:c r="N17" s="38"/>
+      <x:c r="L17" s="39"/>
+      <x:c r="M17" s="37"/>
+      <x:c r="N17" s="37"/>
+      <x:c r="O17" s="37"/>
+      <x:c r="P17" s="37"/>
+      <x:c r="Q17" s="38"/>
+      <x:c r="R17" s="38"/>
+      <x:c r="S17" s="38"/>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="37"/>
@@ -14931,9 +15036,14 @@
       <x:c r="I18" s="37"/>
       <x:c r="J18" s="37"/>
       <x:c r="K18" s="40"/>
-      <x:c r="L18" s="38"/>
-      <x:c r="M18" s="38"/>
-      <x:c r="N18" s="38"/>
+      <x:c r="L18" s="39"/>
+      <x:c r="M18" s="37"/>
+      <x:c r="N18" s="37"/>
+      <x:c r="O18" s="37"/>
+      <x:c r="P18" s="37"/>
+      <x:c r="Q18" s="38"/>
+      <x:c r="R18" s="38"/>
+      <x:c r="S18" s="38"/>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="37"/>
@@ -14947,9 +15057,14 @@
       <x:c r="I19" s="37"/>
       <x:c r="J19" s="37"/>
       <x:c r="K19" s="40"/>
-      <x:c r="L19" s="38"/>
-      <x:c r="M19" s="38"/>
-      <x:c r="N19" s="38"/>
+      <x:c r="L19" s="39"/>
+      <x:c r="M19" s="37"/>
+      <x:c r="N19" s="37"/>
+      <x:c r="O19" s="37"/>
+      <x:c r="P19" s="37"/>
+      <x:c r="Q19" s="38"/>
+      <x:c r="R19" s="38"/>
+      <x:c r="S19" s="38"/>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
       <x:c r="A20" s="37"/>
@@ -14963,9 +15078,14 @@
       <x:c r="I20" s="37"/>
       <x:c r="J20" s="37"/>
       <x:c r="K20" s="40"/>
-      <x:c r="L20" s="38"/>
-      <x:c r="M20" s="38"/>
-      <x:c r="N20" s="38"/>
+      <x:c r="L20" s="39"/>
+      <x:c r="M20" s="37"/>
+      <x:c r="N20" s="37"/>
+      <x:c r="O20" s="37"/>
+      <x:c r="P20" s="37"/>
+      <x:c r="Q20" s="38"/>
+      <x:c r="R20" s="38"/>
+      <x:c r="S20" s="38"/>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="37"/>
@@ -14979,9 +15099,14 @@
       <x:c r="I21" s="37"/>
       <x:c r="J21" s="37"/>
       <x:c r="K21" s="40"/>
-      <x:c r="L21" s="38"/>
-      <x:c r="M21" s="38"/>
-      <x:c r="N21" s="38"/>
+      <x:c r="L21" s="39"/>
+      <x:c r="M21" s="37"/>
+      <x:c r="N21" s="37"/>
+      <x:c r="O21" s="37"/>
+      <x:c r="P21" s="37"/>
+      <x:c r="Q21" s="38"/>
+      <x:c r="R21" s="38"/>
+      <x:c r="S21" s="38"/>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="37"/>
@@ -14995,9 +15120,14 @@
       <x:c r="I22" s="37"/>
       <x:c r="J22" s="37"/>
       <x:c r="K22" s="40"/>
-      <x:c r="L22" s="38"/>
-      <x:c r="M22" s="38"/>
-      <x:c r="N22" s="38"/>
+      <x:c r="L22" s="39"/>
+      <x:c r="M22" s="37"/>
+      <x:c r="N22" s="37"/>
+      <x:c r="O22" s="37"/>
+      <x:c r="P22" s="37"/>
+      <x:c r="Q22" s="38"/>
+      <x:c r="R22" s="38"/>
+      <x:c r="S22" s="38"/>
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
       <x:c r="A23" s="37"/>
@@ -15011,9 +15141,14 @@
       <x:c r="I23" s="37"/>
       <x:c r="J23" s="37"/>
       <x:c r="K23" s="40"/>
-      <x:c r="L23" s="38"/>
-      <x:c r="M23" s="38"/>
-      <x:c r="N23" s="38"/>
+      <x:c r="L23" s="39"/>
+      <x:c r="M23" s="37"/>
+      <x:c r="N23" s="37"/>
+      <x:c r="O23" s="37"/>
+      <x:c r="P23" s="37"/>
+      <x:c r="Q23" s="38"/>
+      <x:c r="R23" s="38"/>
+      <x:c r="S23" s="38"/>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="37"/>
@@ -15027,9 +15162,14 @@
       <x:c r="I24" s="37"/>
       <x:c r="J24" s="37"/>
       <x:c r="K24" s="40"/>
-      <x:c r="L24" s="38"/>
-      <x:c r="M24" s="38"/>
-      <x:c r="N24" s="38"/>
+      <x:c r="L24" s="39"/>
+      <x:c r="M24" s="37"/>
+      <x:c r="N24" s="37"/>
+      <x:c r="O24" s="37"/>
+      <x:c r="P24" s="37"/>
+      <x:c r="Q24" s="38"/>
+      <x:c r="R24" s="38"/>
+      <x:c r="S24" s="38"/>
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
       <x:c r="A25" s="37"/>
@@ -15043,9 +15183,14 @@
       <x:c r="I25" s="37"/>
       <x:c r="J25" s="37"/>
       <x:c r="K25" s="40"/>
-      <x:c r="L25" s="38"/>
-      <x:c r="M25" s="38"/>
-      <x:c r="N25" s="38"/>
+      <x:c r="L25" s="39"/>
+      <x:c r="M25" s="37"/>
+      <x:c r="N25" s="37"/>
+      <x:c r="O25" s="37"/>
+      <x:c r="P25" s="37"/>
+      <x:c r="Q25" s="38"/>
+      <x:c r="R25" s="38"/>
+      <x:c r="S25" s="38"/>
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
       <x:c r="A26" s="37"/>
@@ -15059,9 +15204,14 @@
       <x:c r="I26" s="37"/>
       <x:c r="J26" s="37"/>
       <x:c r="K26" s="40"/>
-      <x:c r="L26" s="38"/>
-      <x:c r="M26" s="38"/>
-      <x:c r="N26" s="38"/>
+      <x:c r="L26" s="39"/>
+      <x:c r="M26" s="37"/>
+      <x:c r="N26" s="37"/>
+      <x:c r="O26" s="37"/>
+      <x:c r="P26" s="37"/>
+      <x:c r="Q26" s="38"/>
+      <x:c r="R26" s="38"/>
+      <x:c r="S26" s="38"/>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="37"/>
@@ -15075,9 +15225,14 @@
       <x:c r="I27" s="37"/>
       <x:c r="J27" s="37"/>
       <x:c r="K27" s="40"/>
-      <x:c r="L27" s="38"/>
-      <x:c r="M27" s="38"/>
-      <x:c r="N27" s="38"/>
+      <x:c r="L27" s="39"/>
+      <x:c r="M27" s="37"/>
+      <x:c r="N27" s="37"/>
+      <x:c r="O27" s="37"/>
+      <x:c r="P27" s="37"/>
+      <x:c r="Q27" s="38"/>
+      <x:c r="R27" s="38"/>
+      <x:c r="S27" s="38"/>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
       <x:c r="A28" s="37"/>
@@ -15091,9 +15246,14 @@
       <x:c r="I28" s="37"/>
       <x:c r="J28" s="37"/>
       <x:c r="K28" s="40"/>
-      <x:c r="L28" s="38"/>
-      <x:c r="M28" s="38"/>
-      <x:c r="N28" s="38"/>
+      <x:c r="L28" s="39"/>
+      <x:c r="M28" s="37"/>
+      <x:c r="N28" s="37"/>
+      <x:c r="O28" s="37"/>
+      <x:c r="P28" s="37"/>
+      <x:c r="Q28" s="38"/>
+      <x:c r="R28" s="38"/>
+      <x:c r="S28" s="38"/>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
       <x:c r="A29" s="37"/>
@@ -15107,9 +15267,14 @@
       <x:c r="I29" s="37"/>
       <x:c r="J29" s="37"/>
       <x:c r="K29" s="40"/>
-      <x:c r="L29" s="38"/>
-      <x:c r="M29" s="38"/>
-      <x:c r="N29" s="38"/>
+      <x:c r="L29" s="39"/>
+      <x:c r="M29" s="37"/>
+      <x:c r="N29" s="37"/>
+      <x:c r="O29" s="37"/>
+      <x:c r="P29" s="37"/>
+      <x:c r="Q29" s="38"/>
+      <x:c r="R29" s="38"/>
+      <x:c r="S29" s="38"/>
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
       <x:c r="A30" s="37"/>
@@ -15123,9 +15288,14 @@
       <x:c r="I30" s="37"/>
       <x:c r="J30" s="37"/>
       <x:c r="K30" s="40"/>
-      <x:c r="L30" s="38"/>
-      <x:c r="M30" s="38"/>
-      <x:c r="N30" s="38"/>
+      <x:c r="L30" s="39"/>
+      <x:c r="M30" s="37"/>
+      <x:c r="N30" s="37"/>
+      <x:c r="O30" s="37"/>
+      <x:c r="P30" s="37"/>
+      <x:c r="Q30" s="38"/>
+      <x:c r="R30" s="38"/>
+      <x:c r="S30" s="38"/>
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
       <x:c r="A31" s="37"/>
@@ -15139,9 +15309,14 @@
       <x:c r="I31" s="37"/>
       <x:c r="J31" s="37"/>
       <x:c r="K31" s="40"/>
-      <x:c r="L31" s="38"/>
-      <x:c r="M31" s="38"/>
-      <x:c r="N31" s="38"/>
+      <x:c r="L31" s="39"/>
+      <x:c r="M31" s="37"/>
+      <x:c r="N31" s="37"/>
+      <x:c r="O31" s="37"/>
+      <x:c r="P31" s="37"/>
+      <x:c r="Q31" s="38"/>
+      <x:c r="R31" s="38"/>
+      <x:c r="S31" s="38"/>
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
       <x:c r="A32" s="37"/>
@@ -15155,9 +15330,14 @@
       <x:c r="I32" s="37"/>
       <x:c r="J32" s="37"/>
       <x:c r="K32" s="40"/>
-      <x:c r="L32" s="38"/>
-      <x:c r="M32" s="38"/>
-      <x:c r="N32" s="38"/>
+      <x:c r="L32" s="39"/>
+      <x:c r="M32" s="37"/>
+      <x:c r="N32" s="37"/>
+      <x:c r="O32" s="37"/>
+      <x:c r="P32" s="37"/>
+      <x:c r="Q32" s="38"/>
+      <x:c r="R32" s="38"/>
+      <x:c r="S32" s="38"/>
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
       <x:c r="A33" s="37"/>
@@ -15171,9 +15351,14 @@
       <x:c r="I33" s="37"/>
       <x:c r="J33" s="37"/>
       <x:c r="K33" s="40"/>
-      <x:c r="L33" s="38"/>
-      <x:c r="M33" s="38"/>
-      <x:c r="N33" s="38"/>
+      <x:c r="L33" s="39"/>
+      <x:c r="M33" s="37"/>
+      <x:c r="N33" s="37"/>
+      <x:c r="O33" s="37"/>
+      <x:c r="P33" s="37"/>
+      <x:c r="Q33" s="38"/>
+      <x:c r="R33" s="38"/>
+      <x:c r="S33" s="38"/>
     </x:row>
     <x:row r="34" ht="24" customHeight="1">
       <x:c r="A34" s="37"/>
@@ -15187,9 +15372,14 @@
       <x:c r="I34" s="37"/>
       <x:c r="J34" s="37"/>
       <x:c r="K34" s="40"/>
-      <x:c r="L34" s="38"/>
-      <x:c r="M34" s="38"/>
-      <x:c r="N34" s="38"/>
+      <x:c r="L34" s="39"/>
+      <x:c r="M34" s="37"/>
+      <x:c r="N34" s="37"/>
+      <x:c r="O34" s="37"/>
+      <x:c r="P34" s="37"/>
+      <x:c r="Q34" s="38"/>
+      <x:c r="R34" s="38"/>
+      <x:c r="S34" s="38"/>
     </x:row>
     <x:row r="35" ht="24" customHeight="1">
       <x:c r="A35" s="37"/>
@@ -15203,9 +15393,14 @@
       <x:c r="I35" s="37"/>
       <x:c r="J35" s="37"/>
       <x:c r="K35" s="40"/>
-      <x:c r="L35" s="38"/>
-      <x:c r="M35" s="38"/>
-      <x:c r="N35" s="38"/>
+      <x:c r="L35" s="39"/>
+      <x:c r="M35" s="37"/>
+      <x:c r="N35" s="37"/>
+      <x:c r="O35" s="37"/>
+      <x:c r="P35" s="37"/>
+      <x:c r="Q35" s="38"/>
+      <x:c r="R35" s="38"/>
+      <x:c r="S35" s="38"/>
     </x:row>
     <x:row r="36" ht="24" customHeight="1">
       <x:c r="A36" s="37"/>
@@ -15219,9 +15414,14 @@
       <x:c r="I36" s="37"/>
       <x:c r="J36" s="37"/>
       <x:c r="K36" s="40"/>
-      <x:c r="L36" s="38"/>
-      <x:c r="M36" s="38"/>
-      <x:c r="N36" s="38"/>
+      <x:c r="L36" s="39"/>
+      <x:c r="M36" s="37"/>
+      <x:c r="N36" s="37"/>
+      <x:c r="O36" s="37"/>
+      <x:c r="P36" s="37"/>
+      <x:c r="Q36" s="38"/>
+      <x:c r="R36" s="38"/>
+      <x:c r="S36" s="38"/>
     </x:row>
     <x:row r="37" ht="24" customHeight="1">
       <x:c r="A37" s="37"/>
@@ -15235,9 +15435,14 @@
       <x:c r="I37" s="37"/>
       <x:c r="J37" s="37"/>
       <x:c r="K37" s="40"/>
-      <x:c r="L37" s="38"/>
-      <x:c r="M37" s="38"/>
-      <x:c r="N37" s="38"/>
+      <x:c r="L37" s="39"/>
+      <x:c r="M37" s="37"/>
+      <x:c r="N37" s="37"/>
+      <x:c r="O37" s="37"/>
+      <x:c r="P37" s="37"/>
+      <x:c r="Q37" s="38"/>
+      <x:c r="R37" s="38"/>
+      <x:c r="S37" s="38"/>
     </x:row>
     <x:row r="38" ht="24" customHeight="1">
       <x:c r="A38" s="37"/>
@@ -15251,9 +15456,14 @@
       <x:c r="I38" s="37"/>
       <x:c r="J38" s="37"/>
       <x:c r="K38" s="40"/>
-      <x:c r="L38" s="38"/>
-      <x:c r="M38" s="38"/>
-      <x:c r="N38" s="38"/>
+      <x:c r="L38" s="39"/>
+      <x:c r="M38" s="37"/>
+      <x:c r="N38" s="37"/>
+      <x:c r="O38" s="37"/>
+      <x:c r="P38" s="37"/>
+      <x:c r="Q38" s="38"/>
+      <x:c r="R38" s="38"/>
+      <x:c r="S38" s="38"/>
     </x:row>
     <x:row r="39" ht="24" customHeight="1">
       <x:c r="A39" s="37"/>
@@ -15267,9 +15477,14 @@
       <x:c r="I39" s="37"/>
       <x:c r="J39" s="37"/>
       <x:c r="K39" s="40"/>
-      <x:c r="L39" s="38"/>
-      <x:c r="M39" s="38"/>
-      <x:c r="N39" s="38"/>
+      <x:c r="L39" s="39"/>
+      <x:c r="M39" s="37"/>
+      <x:c r="N39" s="37"/>
+      <x:c r="O39" s="37"/>
+      <x:c r="P39" s="37"/>
+      <x:c r="Q39" s="38"/>
+      <x:c r="R39" s="38"/>
+      <x:c r="S39" s="38"/>
     </x:row>
     <x:row r="40" ht="24" customHeight="1">
       <x:c r="A40" s="37"/>
@@ -15283,9 +15498,14 @@
       <x:c r="I40" s="37"/>
       <x:c r="J40" s="37"/>
       <x:c r="K40" s="40"/>
-      <x:c r="L40" s="38"/>
-      <x:c r="M40" s="38"/>
-      <x:c r="N40" s="38"/>
+      <x:c r="L40" s="39"/>
+      <x:c r="M40" s="37"/>
+      <x:c r="N40" s="37"/>
+      <x:c r="O40" s="37"/>
+      <x:c r="P40" s="37"/>
+      <x:c r="Q40" s="38"/>
+      <x:c r="R40" s="38"/>
+      <x:c r="S40" s="38"/>
     </x:row>
     <x:row r="41" ht="24" customHeight="1">
       <x:c r="A41" s="37"/>
@@ -15299,9 +15519,14 @@
       <x:c r="I41" s="37"/>
       <x:c r="J41" s="37"/>
       <x:c r="K41" s="40"/>
-      <x:c r="L41" s="38"/>
-      <x:c r="M41" s="38"/>
-      <x:c r="N41" s="38"/>
+      <x:c r="L41" s="39"/>
+      <x:c r="M41" s="37"/>
+      <x:c r="N41" s="37"/>
+      <x:c r="O41" s="37"/>
+      <x:c r="P41" s="37"/>
+      <x:c r="Q41" s="38"/>
+      <x:c r="R41" s="38"/>
+      <x:c r="S41" s="38"/>
     </x:row>
     <x:row r="42" ht="24" customHeight="1">
       <x:c r="A42" s="37"/>
@@ -15315,9 +15540,14 @@
       <x:c r="I42" s="37"/>
       <x:c r="J42" s="37"/>
       <x:c r="K42" s="40"/>
-      <x:c r="L42" s="38"/>
-      <x:c r="M42" s="38"/>
-      <x:c r="N42" s="38"/>
+      <x:c r="L42" s="39"/>
+      <x:c r="M42" s="37"/>
+      <x:c r="N42" s="37"/>
+      <x:c r="O42" s="37"/>
+      <x:c r="P42" s="37"/>
+      <x:c r="Q42" s="38"/>
+      <x:c r="R42" s="38"/>
+      <x:c r="S42" s="38"/>
     </x:row>
     <x:row r="43" ht="24" customHeight="1">
       <x:c r="A43" s="37"/>
@@ -15331,9 +15561,14 @@
       <x:c r="I43" s="37"/>
       <x:c r="J43" s="37"/>
       <x:c r="K43" s="40"/>
-      <x:c r="L43" s="38"/>
-      <x:c r="M43" s="38"/>
-      <x:c r="N43" s="38"/>
+      <x:c r="L43" s="39"/>
+      <x:c r="M43" s="37"/>
+      <x:c r="N43" s="37"/>
+      <x:c r="O43" s="37"/>
+      <x:c r="P43" s="37"/>
+      <x:c r="Q43" s="38"/>
+      <x:c r="R43" s="38"/>
+      <x:c r="S43" s="38"/>
     </x:row>
     <x:row r="44" ht="24" customHeight="1">
       <x:c r="A44" s="37"/>
@@ -15347,9 +15582,14 @@
       <x:c r="I44" s="37"/>
       <x:c r="J44" s="37"/>
       <x:c r="K44" s="40"/>
-      <x:c r="L44" s="38"/>
-      <x:c r="M44" s="38"/>
-      <x:c r="N44" s="38"/>
+      <x:c r="L44" s="39"/>
+      <x:c r="M44" s="37"/>
+      <x:c r="N44" s="37"/>
+      <x:c r="O44" s="37"/>
+      <x:c r="P44" s="37"/>
+      <x:c r="Q44" s="38"/>
+      <x:c r="R44" s="38"/>
+      <x:c r="S44" s="38"/>
     </x:row>
     <x:row r="45" ht="24" customHeight="1">
       <x:c r="A45" s="37"/>
@@ -15363,9 +15603,14 @@
       <x:c r="I45" s="37"/>
       <x:c r="J45" s="37"/>
       <x:c r="K45" s="40"/>
-      <x:c r="L45" s="38"/>
-      <x:c r="M45" s="38"/>
-      <x:c r="N45" s="38"/>
+      <x:c r="L45" s="39"/>
+      <x:c r="M45" s="37"/>
+      <x:c r="N45" s="37"/>
+      <x:c r="O45" s="37"/>
+      <x:c r="P45" s="37"/>
+      <x:c r="Q45" s="38"/>
+      <x:c r="R45" s="38"/>
+      <x:c r="S45" s="38"/>
     </x:row>
     <x:row r="46" ht="24" customHeight="1">
       <x:c r="A46" s="37"/>
@@ -15379,9 +15624,14 @@
       <x:c r="I46" s="37"/>
       <x:c r="J46" s="37"/>
       <x:c r="K46" s="40"/>
-      <x:c r="L46" s="38"/>
-      <x:c r="M46" s="38"/>
-      <x:c r="N46" s="38"/>
+      <x:c r="L46" s="39"/>
+      <x:c r="M46" s="37"/>
+      <x:c r="N46" s="37"/>
+      <x:c r="O46" s="37"/>
+      <x:c r="P46" s="37"/>
+      <x:c r="Q46" s="38"/>
+      <x:c r="R46" s="38"/>
+      <x:c r="S46" s="38"/>
     </x:row>
     <x:row r="47" ht="24" customHeight="1">
       <x:c r="A47" s="37"/>
@@ -15395,9 +15645,14 @@
       <x:c r="I47" s="37"/>
       <x:c r="J47" s="37"/>
       <x:c r="K47" s="40"/>
-      <x:c r="L47" s="38"/>
-      <x:c r="M47" s="38"/>
-      <x:c r="N47" s="38"/>
+      <x:c r="L47" s="39"/>
+      <x:c r="M47" s="37"/>
+      <x:c r="N47" s="37"/>
+      <x:c r="O47" s="37"/>
+      <x:c r="P47" s="37"/>
+      <x:c r="Q47" s="38"/>
+      <x:c r="R47" s="38"/>
+      <x:c r="S47" s="38"/>
     </x:row>
     <x:row r="48" ht="24" customHeight="1">
       <x:c r="A48" s="37"/>
@@ -15411,9 +15666,14 @@
       <x:c r="I48" s="37"/>
       <x:c r="J48" s="37"/>
       <x:c r="K48" s="40"/>
-      <x:c r="L48" s="38"/>
-      <x:c r="M48" s="38"/>
-      <x:c r="N48" s="38"/>
+      <x:c r="L48" s="39"/>
+      <x:c r="M48" s="37"/>
+      <x:c r="N48" s="37"/>
+      <x:c r="O48" s="37"/>
+      <x:c r="P48" s="37"/>
+      <x:c r="Q48" s="38"/>
+      <x:c r="R48" s="38"/>
+      <x:c r="S48" s="38"/>
     </x:row>
     <x:row r="49" ht="24" customHeight="1">
       <x:c r="A49" s="37"/>
@@ -15427,9 +15687,14 @@
       <x:c r="I49" s="37"/>
       <x:c r="J49" s="37"/>
       <x:c r="K49" s="40"/>
-      <x:c r="L49" s="38"/>
-      <x:c r="M49" s="38"/>
-      <x:c r="N49" s="38"/>
+      <x:c r="L49" s="39"/>
+      <x:c r="M49" s="37"/>
+      <x:c r="N49" s="37"/>
+      <x:c r="O49" s="37"/>
+      <x:c r="P49" s="37"/>
+      <x:c r="Q49" s="38"/>
+      <x:c r="R49" s="38"/>
+      <x:c r="S49" s="38"/>
     </x:row>
     <x:row r="50" ht="24" customHeight="1">
       <x:c r="A50" s="37"/>
@@ -15443,9 +15708,14 @@
       <x:c r="I50" s="37"/>
       <x:c r="J50" s="37"/>
       <x:c r="K50" s="40"/>
-      <x:c r="L50" s="38"/>
-      <x:c r="M50" s="38"/>
-      <x:c r="N50" s="38"/>
+      <x:c r="L50" s="39"/>
+      <x:c r="M50" s="37"/>
+      <x:c r="N50" s="37"/>
+      <x:c r="O50" s="37"/>
+      <x:c r="P50" s="37"/>
+      <x:c r="Q50" s="38"/>
+      <x:c r="R50" s="38"/>
+      <x:c r="S50" s="38"/>
     </x:row>
     <x:row r="51" ht="24" customHeight="1">
       <x:c r="A51" s="37"/>
@@ -15459,9 +15729,14 @@
       <x:c r="I51" s="37"/>
       <x:c r="J51" s="37"/>
       <x:c r="K51" s="40"/>
-      <x:c r="L51" s="38"/>
-      <x:c r="M51" s="38"/>
-      <x:c r="N51" s="38"/>
+      <x:c r="L51" s="39"/>
+      <x:c r="M51" s="37"/>
+      <x:c r="N51" s="37"/>
+      <x:c r="O51" s="37"/>
+      <x:c r="P51" s="37"/>
+      <x:c r="Q51" s="38"/>
+      <x:c r="R51" s="38"/>
+      <x:c r="S51" s="38"/>
     </x:row>
     <x:row r="52" ht="24" customHeight="1">
       <x:c r="A52" s="37"/>
@@ -15475,9 +15750,14 @@
       <x:c r="I52" s="37"/>
       <x:c r="J52" s="37"/>
       <x:c r="K52" s="40"/>
-      <x:c r="L52" s="38"/>
-      <x:c r="M52" s="38"/>
-      <x:c r="N52" s="38"/>
+      <x:c r="L52" s="39"/>
+      <x:c r="M52" s="37"/>
+      <x:c r="N52" s="37"/>
+      <x:c r="O52" s="37"/>
+      <x:c r="P52" s="37"/>
+      <x:c r="Q52" s="38"/>
+      <x:c r="R52" s="38"/>
+      <x:c r="S52" s="38"/>
     </x:row>
     <x:row r="53" ht="24" customHeight="1">
       <x:c r="A53" s="37"/>
@@ -15491,9 +15771,14 @@
       <x:c r="I53" s="37"/>
       <x:c r="J53" s="37"/>
       <x:c r="K53" s="40"/>
-      <x:c r="L53" s="38"/>
-      <x:c r="M53" s="38"/>
-      <x:c r="N53" s="38"/>
+      <x:c r="L53" s="39"/>
+      <x:c r="M53" s="37"/>
+      <x:c r="N53" s="37"/>
+      <x:c r="O53" s="37"/>
+      <x:c r="P53" s="37"/>
+      <x:c r="Q53" s="38"/>
+      <x:c r="R53" s="38"/>
+      <x:c r="S53" s="38"/>
     </x:row>
     <x:row r="54" ht="24" customHeight="1">
       <x:c r="A54" s="37"/>
@@ -15507,9 +15792,14 @@
       <x:c r="I54" s="37"/>
       <x:c r="J54" s="37"/>
       <x:c r="K54" s="40"/>
-      <x:c r="L54" s="38"/>
-      <x:c r="M54" s="38"/>
-      <x:c r="N54" s="38"/>
+      <x:c r="L54" s="39"/>
+      <x:c r="M54" s="37"/>
+      <x:c r="N54" s="37"/>
+      <x:c r="O54" s="37"/>
+      <x:c r="P54" s="37"/>
+      <x:c r="Q54" s="38"/>
+      <x:c r="R54" s="38"/>
+      <x:c r="S54" s="38"/>
     </x:row>
     <x:row r="55" ht="24" customHeight="1">
       <x:c r="A55" s="37"/>
@@ -15523,9 +15813,14 @@
       <x:c r="I55" s="37"/>
       <x:c r="J55" s="37"/>
       <x:c r="K55" s="40"/>
-      <x:c r="L55" s="38"/>
-      <x:c r="M55" s="38"/>
-      <x:c r="N55" s="38"/>
+      <x:c r="L55" s="39"/>
+      <x:c r="M55" s="37"/>
+      <x:c r="N55" s="37"/>
+      <x:c r="O55" s="37"/>
+      <x:c r="P55" s="37"/>
+      <x:c r="Q55" s="38"/>
+      <x:c r="R55" s="38"/>
+      <x:c r="S55" s="38"/>
     </x:row>
     <x:row r="56" ht="24" customHeight="1">
       <x:c r="A56" s="37"/>
@@ -15539,9 +15834,14 @@
       <x:c r="I56" s="37"/>
       <x:c r="J56" s="37"/>
       <x:c r="K56" s="40"/>
-      <x:c r="L56" s="38"/>
-      <x:c r="M56" s="38"/>
-      <x:c r="N56" s="38"/>
+      <x:c r="L56" s="39"/>
+      <x:c r="M56" s="37"/>
+      <x:c r="N56" s="37"/>
+      <x:c r="O56" s="37"/>
+      <x:c r="P56" s="37"/>
+      <x:c r="Q56" s="38"/>
+      <x:c r="R56" s="38"/>
+      <x:c r="S56" s="38"/>
     </x:row>
     <x:row r="57" ht="24" customHeight="1">
       <x:c r="A57" s="37"/>
@@ -15555,9 +15855,14 @@
       <x:c r="I57" s="37"/>
       <x:c r="J57" s="37"/>
       <x:c r="K57" s="40"/>
-      <x:c r="L57" s="38"/>
-      <x:c r="M57" s="38"/>
-      <x:c r="N57" s="38"/>
+      <x:c r="L57" s="39"/>
+      <x:c r="M57" s="37"/>
+      <x:c r="N57" s="37"/>
+      <x:c r="O57" s="37"/>
+      <x:c r="P57" s="37"/>
+      <x:c r="Q57" s="38"/>
+      <x:c r="R57" s="38"/>
+      <x:c r="S57" s="38"/>
     </x:row>
     <x:row r="58" ht="24" customHeight="1">
       <x:c r="A58" s="37"/>
@@ -15571,9 +15876,14 @@
       <x:c r="I58" s="37"/>
       <x:c r="J58" s="37"/>
       <x:c r="K58" s="40"/>
-      <x:c r="L58" s="38"/>
-      <x:c r="M58" s="38"/>
-      <x:c r="N58" s="38"/>
+      <x:c r="L58" s="39"/>
+      <x:c r="M58" s="37"/>
+      <x:c r="N58" s="37"/>
+      <x:c r="O58" s="37"/>
+      <x:c r="P58" s="37"/>
+      <x:c r="Q58" s="38"/>
+      <x:c r="R58" s="38"/>
+      <x:c r="S58" s="38"/>
     </x:row>
     <x:row r="59" ht="24" customHeight="1">
       <x:c r="A59" s="37"/>
@@ -15587,9 +15897,14 @@
       <x:c r="I59" s="37"/>
       <x:c r="J59" s="37"/>
       <x:c r="K59" s="40"/>
-      <x:c r="L59" s="38"/>
-      <x:c r="M59" s="38"/>
-      <x:c r="N59" s="38"/>
+      <x:c r="L59" s="39"/>
+      <x:c r="M59" s="37"/>
+      <x:c r="N59" s="37"/>
+      <x:c r="O59" s="37"/>
+      <x:c r="P59" s="37"/>
+      <x:c r="Q59" s="38"/>
+      <x:c r="R59" s="38"/>
+      <x:c r="S59" s="38"/>
     </x:row>
     <x:row r="60" ht="24" customHeight="1">
       <x:c r="A60" s="37"/>
@@ -15603,9 +15918,14 @@
       <x:c r="I60" s="37"/>
       <x:c r="J60" s="37"/>
       <x:c r="K60" s="40"/>
-      <x:c r="L60" s="38"/>
-      <x:c r="M60" s="38"/>
-      <x:c r="N60" s="38"/>
+      <x:c r="L60" s="39"/>
+      <x:c r="M60" s="37"/>
+      <x:c r="N60" s="37"/>
+      <x:c r="O60" s="37"/>
+      <x:c r="P60" s="37"/>
+      <x:c r="Q60" s="38"/>
+      <x:c r="R60" s="38"/>
+      <x:c r="S60" s="38"/>
     </x:row>
     <x:row r="61" ht="24" customHeight="1">
       <x:c r="A61" s="37"/>
@@ -15619,9 +15939,14 @@
       <x:c r="I61" s="37"/>
       <x:c r="J61" s="37"/>
       <x:c r="K61" s="40"/>
-      <x:c r="L61" s="38"/>
-      <x:c r="M61" s="38"/>
-      <x:c r="N61" s="38"/>
+      <x:c r="L61" s="39"/>
+      <x:c r="M61" s="37"/>
+      <x:c r="N61" s="37"/>
+      <x:c r="O61" s="37"/>
+      <x:c r="P61" s="37"/>
+      <x:c r="Q61" s="38"/>
+      <x:c r="R61" s="38"/>
+      <x:c r="S61" s="38"/>
     </x:row>
     <x:row r="62" ht="24" customHeight="1">
       <x:c r="A62" s="37"/>
@@ -15635,9 +15960,14 @@
       <x:c r="I62" s="37"/>
       <x:c r="J62" s="37"/>
       <x:c r="K62" s="40"/>
-      <x:c r="L62" s="38"/>
-      <x:c r="M62" s="38"/>
-      <x:c r="N62" s="38"/>
+      <x:c r="L62" s="39"/>
+      <x:c r="M62" s="37"/>
+      <x:c r="N62" s="37"/>
+      <x:c r="O62" s="37"/>
+      <x:c r="P62" s="37"/>
+      <x:c r="Q62" s="38"/>
+      <x:c r="R62" s="38"/>
+      <x:c r="S62" s="38"/>
     </x:row>
     <x:row r="63" ht="24" customHeight="1">
       <x:c r="A63" s="37"/>
@@ -15651,9 +15981,14 @@
       <x:c r="I63" s="37"/>
       <x:c r="J63" s="37"/>
       <x:c r="K63" s="40"/>
-      <x:c r="L63" s="38"/>
-      <x:c r="M63" s="38"/>
-      <x:c r="N63" s="38"/>
+      <x:c r="L63" s="39"/>
+      <x:c r="M63" s="37"/>
+      <x:c r="N63" s="37"/>
+      <x:c r="O63" s="37"/>
+      <x:c r="P63" s="37"/>
+      <x:c r="Q63" s="38"/>
+      <x:c r="R63" s="38"/>
+      <x:c r="S63" s="38"/>
     </x:row>
     <x:row r="64" ht="24" customHeight="1">
       <x:c r="A64" s="37"/>
@@ -15667,9 +16002,14 @@
       <x:c r="I64" s="37"/>
       <x:c r="J64" s="37"/>
       <x:c r="K64" s="40"/>
-      <x:c r="L64" s="38"/>
-      <x:c r="M64" s="38"/>
-      <x:c r="N64" s="38"/>
+      <x:c r="L64" s="39"/>
+      <x:c r="M64" s="37"/>
+      <x:c r="N64" s="37"/>
+      <x:c r="O64" s="37"/>
+      <x:c r="P64" s="37"/>
+      <x:c r="Q64" s="38"/>
+      <x:c r="R64" s="38"/>
+      <x:c r="S64" s="38"/>
     </x:row>
     <x:row r="65" ht="24" customHeight="1">
       <x:c r="A65" s="37"/>
@@ -15683,9 +16023,14 @@
       <x:c r="I65" s="37"/>
       <x:c r="J65" s="37"/>
       <x:c r="K65" s="40"/>
-      <x:c r="L65" s="38"/>
-      <x:c r="M65" s="38"/>
-      <x:c r="N65" s="38"/>
+      <x:c r="L65" s="39"/>
+      <x:c r="M65" s="37"/>
+      <x:c r="N65" s="37"/>
+      <x:c r="O65" s="37"/>
+      <x:c r="P65" s="37"/>
+      <x:c r="Q65" s="38"/>
+      <x:c r="R65" s="38"/>
+      <x:c r="S65" s="38"/>
     </x:row>
     <x:row r="66" ht="24" customHeight="1">
       <x:c r="A66" s="37"/>
@@ -15699,9 +16044,14 @@
       <x:c r="I66" s="37"/>
       <x:c r="J66" s="37"/>
       <x:c r="K66" s="40"/>
-      <x:c r="L66" s="38"/>
-      <x:c r="M66" s="38"/>
-      <x:c r="N66" s="38"/>
+      <x:c r="L66" s="39"/>
+      <x:c r="M66" s="37"/>
+      <x:c r="N66" s="37"/>
+      <x:c r="O66" s="37"/>
+      <x:c r="P66" s="37"/>
+      <x:c r="Q66" s="38"/>
+      <x:c r="R66" s="38"/>
+      <x:c r="S66" s="38"/>
     </x:row>
     <x:row r="67" ht="24" customHeight="1">
       <x:c r="A67" s="37"/>
@@ -15715,9 +16065,14 @@
       <x:c r="I67" s="37"/>
       <x:c r="J67" s="37"/>
       <x:c r="K67" s="40"/>
-      <x:c r="L67" s="38"/>
-      <x:c r="M67" s="38"/>
-      <x:c r="N67" s="38"/>
+      <x:c r="L67" s="39"/>
+      <x:c r="M67" s="37"/>
+      <x:c r="N67" s="37"/>
+      <x:c r="O67" s="37"/>
+      <x:c r="P67" s="37"/>
+      <x:c r="Q67" s="38"/>
+      <x:c r="R67" s="38"/>
+      <x:c r="S67" s="38"/>
     </x:row>
     <x:row r="68" ht="24" customHeight="1">
       <x:c r="A68" s="37"/>
@@ -15731,9 +16086,14 @@
       <x:c r="I68" s="37"/>
       <x:c r="J68" s="37"/>
       <x:c r="K68" s="40"/>
-      <x:c r="L68" s="38"/>
-      <x:c r="M68" s="38"/>
-      <x:c r="N68" s="38"/>
+      <x:c r="L68" s="39"/>
+      <x:c r="M68" s="37"/>
+      <x:c r="N68" s="37"/>
+      <x:c r="O68" s="37"/>
+      <x:c r="P68" s="37"/>
+      <x:c r="Q68" s="38"/>
+      <x:c r="R68" s="38"/>
+      <x:c r="S68" s="38"/>
     </x:row>
     <x:row r="69" ht="24" customHeight="1">
       <x:c r="A69" s="37"/>
@@ -15747,9 +16107,14 @@
       <x:c r="I69" s="37"/>
       <x:c r="J69" s="37"/>
       <x:c r="K69" s="40"/>
-      <x:c r="L69" s="38"/>
-      <x:c r="M69" s="38"/>
-      <x:c r="N69" s="38"/>
+      <x:c r="L69" s="39"/>
+      <x:c r="M69" s="37"/>
+      <x:c r="N69" s="37"/>
+      <x:c r="O69" s="37"/>
+      <x:c r="P69" s="37"/>
+      <x:c r="Q69" s="38"/>
+      <x:c r="R69" s="38"/>
+      <x:c r="S69" s="38"/>
     </x:row>
     <x:row r="70" ht="24" customHeight="1">
       <x:c r="A70" s="37"/>
@@ -15763,9 +16128,14 @@
       <x:c r="I70" s="37"/>
       <x:c r="J70" s="37"/>
       <x:c r="K70" s="40"/>
-      <x:c r="L70" s="38"/>
-      <x:c r="M70" s="38"/>
-      <x:c r="N70" s="38"/>
+      <x:c r="L70" s="39"/>
+      <x:c r="M70" s="37"/>
+      <x:c r="N70" s="37"/>
+      <x:c r="O70" s="37"/>
+      <x:c r="P70" s="37"/>
+      <x:c r="Q70" s="38"/>
+      <x:c r="R70" s="38"/>
+      <x:c r="S70" s="38"/>
     </x:row>
     <x:row r="71" ht="24" customHeight="1">
       <x:c r="A71" s="37"/>
@@ -15779,9 +16149,14 @@
       <x:c r="I71" s="37"/>
       <x:c r="J71" s="37"/>
       <x:c r="K71" s="40"/>
-      <x:c r="L71" s="38"/>
-      <x:c r="M71" s="38"/>
-      <x:c r="N71" s="38"/>
+      <x:c r="L71" s="39"/>
+      <x:c r="M71" s="37"/>
+      <x:c r="N71" s="37"/>
+      <x:c r="O71" s="37"/>
+      <x:c r="P71" s="37"/>
+      <x:c r="Q71" s="38"/>
+      <x:c r="R71" s="38"/>
+      <x:c r="S71" s="38"/>
     </x:row>
     <x:row r="72" ht="24" customHeight="1">
       <x:c r="A72" s="37"/>
@@ -15795,9 +16170,14 @@
       <x:c r="I72" s="37"/>
       <x:c r="J72" s="37"/>
       <x:c r="K72" s="40"/>
-      <x:c r="L72" s="38"/>
-      <x:c r="M72" s="38"/>
-      <x:c r="N72" s="38"/>
+      <x:c r="L72" s="39"/>
+      <x:c r="M72" s="37"/>
+      <x:c r="N72" s="37"/>
+      <x:c r="O72" s="37"/>
+      <x:c r="P72" s="37"/>
+      <x:c r="Q72" s="38"/>
+      <x:c r="R72" s="38"/>
+      <x:c r="S72" s="38"/>
     </x:row>
     <x:row r="73" ht="24" customHeight="1">
       <x:c r="A73" s="37"/>
@@ -15811,9 +16191,14 @@
       <x:c r="I73" s="37"/>
       <x:c r="J73" s="37"/>
       <x:c r="K73" s="40"/>
-      <x:c r="L73" s="38"/>
-      <x:c r="M73" s="38"/>
-      <x:c r="N73" s="38"/>
+      <x:c r="L73" s="39"/>
+      <x:c r="M73" s="37"/>
+      <x:c r="N73" s="37"/>
+      <x:c r="O73" s="37"/>
+      <x:c r="P73" s="37"/>
+      <x:c r="Q73" s="38"/>
+      <x:c r="R73" s="38"/>
+      <x:c r="S73" s="38"/>
     </x:row>
     <x:row r="74" ht="24" customHeight="1">
       <x:c r="A74" s="37"/>
@@ -15827,9 +16212,14 @@
       <x:c r="I74" s="37"/>
       <x:c r="J74" s="37"/>
       <x:c r="K74" s="40"/>
-      <x:c r="L74" s="38"/>
-      <x:c r="M74" s="38"/>
-      <x:c r="N74" s="38"/>
+      <x:c r="L74" s="39"/>
+      <x:c r="M74" s="37"/>
+      <x:c r="N74" s="37"/>
+      <x:c r="O74" s="37"/>
+      <x:c r="P74" s="37"/>
+      <x:c r="Q74" s="38"/>
+      <x:c r="R74" s="38"/>
+      <x:c r="S74" s="38"/>
     </x:row>
     <x:row r="75" ht="24" customHeight="1">
       <x:c r="A75" s="37"/>
@@ -15843,9 +16233,14 @@
       <x:c r="I75" s="37"/>
       <x:c r="J75" s="37"/>
       <x:c r="K75" s="40"/>
-      <x:c r="L75" s="38"/>
-      <x:c r="M75" s="38"/>
-      <x:c r="N75" s="38"/>
+      <x:c r="L75" s="39"/>
+      <x:c r="M75" s="37"/>
+      <x:c r="N75" s="37"/>
+      <x:c r="O75" s="37"/>
+      <x:c r="P75" s="37"/>
+      <x:c r="Q75" s="38"/>
+      <x:c r="R75" s="38"/>
+      <x:c r="S75" s="38"/>
     </x:row>
     <x:row r="76" ht="24" customHeight="1">
       <x:c r="A76" s="37"/>
@@ -15859,9 +16254,14 @@
       <x:c r="I76" s="37"/>
       <x:c r="J76" s="37"/>
       <x:c r="K76" s="40"/>
-      <x:c r="L76" s="38"/>
-      <x:c r="M76" s="38"/>
-      <x:c r="N76" s="38"/>
+      <x:c r="L76" s="39"/>
+      <x:c r="M76" s="37"/>
+      <x:c r="N76" s="37"/>
+      <x:c r="O76" s="37"/>
+      <x:c r="P76" s="37"/>
+      <x:c r="Q76" s="38"/>
+      <x:c r="R76" s="38"/>
+      <x:c r="S76" s="38"/>
     </x:row>
     <x:row r="77" ht="24" customHeight="1">
       <x:c r="A77" s="37"/>
@@ -15875,9 +16275,14 @@
       <x:c r="I77" s="37"/>
       <x:c r="J77" s="37"/>
       <x:c r="K77" s="40"/>
-      <x:c r="L77" s="38"/>
-      <x:c r="M77" s="38"/>
-      <x:c r="N77" s="38"/>
+      <x:c r="L77" s="39"/>
+      <x:c r="M77" s="37"/>
+      <x:c r="N77" s="37"/>
+      <x:c r="O77" s="37"/>
+      <x:c r="P77" s="37"/>
+      <x:c r="Q77" s="38"/>
+      <x:c r="R77" s="38"/>
+      <x:c r="S77" s="38"/>
     </x:row>
     <x:row r="78" ht="24" customHeight="1">
       <x:c r="A78" s="37"/>
@@ -15891,9 +16296,14 @@
       <x:c r="I78" s="37"/>
       <x:c r="J78" s="37"/>
       <x:c r="K78" s="40"/>
-      <x:c r="L78" s="38"/>
-      <x:c r="M78" s="38"/>
-      <x:c r="N78" s="38"/>
+      <x:c r="L78" s="39"/>
+      <x:c r="M78" s="37"/>
+      <x:c r="N78" s="37"/>
+      <x:c r="O78" s="37"/>
+      <x:c r="P78" s="37"/>
+      <x:c r="Q78" s="38"/>
+      <x:c r="R78" s="38"/>
+      <x:c r="S78" s="38"/>
     </x:row>
     <x:row r="79" ht="24" customHeight="1">
       <x:c r="A79" s="37"/>
@@ -15907,9 +16317,14 @@
       <x:c r="I79" s="37"/>
       <x:c r="J79" s="37"/>
       <x:c r="K79" s="40"/>
-      <x:c r="L79" s="38"/>
-      <x:c r="M79" s="38"/>
-      <x:c r="N79" s="38"/>
+      <x:c r="L79" s="39"/>
+      <x:c r="M79" s="37"/>
+      <x:c r="N79" s="37"/>
+      <x:c r="O79" s="37"/>
+      <x:c r="P79" s="37"/>
+      <x:c r="Q79" s="38"/>
+      <x:c r="R79" s="38"/>
+      <x:c r="S79" s="38"/>
     </x:row>
     <x:row r="80" ht="24" customHeight="1">
       <x:c r="A80" s="37"/>
@@ -15923,9 +16338,14 @@
       <x:c r="I80" s="37"/>
       <x:c r="J80" s="37"/>
       <x:c r="K80" s="40"/>
-      <x:c r="L80" s="38"/>
-      <x:c r="M80" s="38"/>
-      <x:c r="N80" s="38"/>
+      <x:c r="L80" s="39"/>
+      <x:c r="M80" s="37"/>
+      <x:c r="N80" s="37"/>
+      <x:c r="O80" s="37"/>
+      <x:c r="P80" s="37"/>
+      <x:c r="Q80" s="38"/>
+      <x:c r="R80" s="38"/>
+      <x:c r="S80" s="38"/>
     </x:row>
     <x:row r="81" ht="24" customHeight="1">
       <x:c r="A81" s="37"/>
@@ -15939,9 +16359,14 @@
       <x:c r="I81" s="37"/>
       <x:c r="J81" s="37"/>
       <x:c r="K81" s="40"/>
-      <x:c r="L81" s="38"/>
-      <x:c r="M81" s="38"/>
-      <x:c r="N81" s="38"/>
+      <x:c r="L81" s="39"/>
+      <x:c r="M81" s="37"/>
+      <x:c r="N81" s="37"/>
+      <x:c r="O81" s="37"/>
+      <x:c r="P81" s="37"/>
+      <x:c r="Q81" s="38"/>
+      <x:c r="R81" s="38"/>
+      <x:c r="S81" s="38"/>
     </x:row>
     <x:row r="82" ht="24" customHeight="1">
       <x:c r="A82" s="37"/>
@@ -15955,9 +16380,14 @@
       <x:c r="I82" s="37"/>
       <x:c r="J82" s="37"/>
       <x:c r="K82" s="40"/>
-      <x:c r="L82" s="38"/>
-      <x:c r="M82" s="38"/>
-      <x:c r="N82" s="38"/>
+      <x:c r="L82" s="39"/>
+      <x:c r="M82" s="37"/>
+      <x:c r="N82" s="37"/>
+      <x:c r="O82" s="37"/>
+      <x:c r="P82" s="37"/>
+      <x:c r="Q82" s="38"/>
+      <x:c r="R82" s="38"/>
+      <x:c r="S82" s="38"/>
     </x:row>
     <x:row r="83" ht="24" customHeight="1">
       <x:c r="A83" s="37"/>
@@ -15971,9 +16401,14 @@
       <x:c r="I83" s="37"/>
       <x:c r="J83" s="37"/>
       <x:c r="K83" s="40"/>
-      <x:c r="L83" s="38"/>
-      <x:c r="M83" s="38"/>
-      <x:c r="N83" s="38"/>
+      <x:c r="L83" s="39"/>
+      <x:c r="M83" s="37"/>
+      <x:c r="N83" s="37"/>
+      <x:c r="O83" s="37"/>
+      <x:c r="P83" s="37"/>
+      <x:c r="Q83" s="38"/>
+      <x:c r="R83" s="38"/>
+      <x:c r="S83" s="38"/>
     </x:row>
     <x:row r="84" ht="24" customHeight="1">
       <x:c r="A84" s="37"/>
@@ -15987,9 +16422,14 @@
       <x:c r="I84" s="37"/>
       <x:c r="J84" s="37"/>
       <x:c r="K84" s="40"/>
-      <x:c r="L84" s="38"/>
-      <x:c r="M84" s="38"/>
-      <x:c r="N84" s="38"/>
+      <x:c r="L84" s="39"/>
+      <x:c r="M84" s="37"/>
+      <x:c r="N84" s="37"/>
+      <x:c r="O84" s="37"/>
+      <x:c r="P84" s="37"/>
+      <x:c r="Q84" s="38"/>
+      <x:c r="R84" s="38"/>
+      <x:c r="S84" s="38"/>
     </x:row>
     <x:row r="85" ht="24" customHeight="1">
       <x:c r="A85" s="37"/>
@@ -16003,9 +16443,14 @@
       <x:c r="I85" s="37"/>
       <x:c r="J85" s="37"/>
       <x:c r="K85" s="40"/>
-      <x:c r="L85" s="38"/>
-      <x:c r="M85" s="38"/>
-      <x:c r="N85" s="38"/>
+      <x:c r="L85" s="39"/>
+      <x:c r="M85" s="37"/>
+      <x:c r="N85" s="37"/>
+      <x:c r="O85" s="37"/>
+      <x:c r="P85" s="37"/>
+      <x:c r="Q85" s="38"/>
+      <x:c r="R85" s="38"/>
+      <x:c r="S85" s="38"/>
     </x:row>
     <x:row r="86" ht="24" customHeight="1">
       <x:c r="A86" s="37"/>
@@ -16019,9 +16464,14 @@
       <x:c r="I86" s="37"/>
       <x:c r="J86" s="37"/>
       <x:c r="K86" s="40"/>
-      <x:c r="L86" s="38"/>
-      <x:c r="M86" s="38"/>
-      <x:c r="N86" s="38"/>
+      <x:c r="L86" s="39"/>
+      <x:c r="M86" s="37"/>
+      <x:c r="N86" s="37"/>
+      <x:c r="O86" s="37"/>
+      <x:c r="P86" s="37"/>
+      <x:c r="Q86" s="38"/>
+      <x:c r="R86" s="38"/>
+      <x:c r="S86" s="38"/>
     </x:row>
     <x:row r="87" ht="24" customHeight="1">
       <x:c r="A87" s="37"/>
@@ -16035,9 +16485,14 @@
       <x:c r="I87" s="37"/>
       <x:c r="J87" s="37"/>
       <x:c r="K87" s="40"/>
-      <x:c r="L87" s="38"/>
-      <x:c r="M87" s="38"/>
-      <x:c r="N87" s="38"/>
+      <x:c r="L87" s="39"/>
+      <x:c r="M87" s="37"/>
+      <x:c r="N87" s="37"/>
+      <x:c r="O87" s="37"/>
+      <x:c r="P87" s="37"/>
+      <x:c r="Q87" s="38"/>
+      <x:c r="R87" s="38"/>
+      <x:c r="S87" s="38"/>
     </x:row>
     <x:row r="88" ht="24" customHeight="1">
       <x:c r="A88" s="37"/>
@@ -16051,9 +16506,14 @@
       <x:c r="I88" s="37"/>
       <x:c r="J88" s="37"/>
       <x:c r="K88" s="40"/>
-      <x:c r="L88" s="38"/>
-      <x:c r="M88" s="38"/>
-      <x:c r="N88" s="38"/>
+      <x:c r="L88" s="39"/>
+      <x:c r="M88" s="37"/>
+      <x:c r="N88" s="37"/>
+      <x:c r="O88" s="37"/>
+      <x:c r="P88" s="37"/>
+      <x:c r="Q88" s="38"/>
+      <x:c r="R88" s="38"/>
+      <x:c r="S88" s="38"/>
     </x:row>
     <x:row r="89" ht="24" customHeight="1">
       <x:c r="A89" s="37"/>
@@ -16067,9 +16527,14 @@
       <x:c r="I89" s="37"/>
       <x:c r="J89" s="37"/>
       <x:c r="K89" s="40"/>
-      <x:c r="L89" s="38"/>
-      <x:c r="M89" s="38"/>
-      <x:c r="N89" s="38"/>
+      <x:c r="L89" s="39"/>
+      <x:c r="M89" s="37"/>
+      <x:c r="N89" s="37"/>
+      <x:c r="O89" s="37"/>
+      <x:c r="P89" s="37"/>
+      <x:c r="Q89" s="38"/>
+      <x:c r="R89" s="38"/>
+      <x:c r="S89" s="38"/>
     </x:row>
     <x:row r="90" ht="24" customHeight="1">
       <x:c r="A90" s="37"/>
@@ -16083,9 +16548,14 @@
       <x:c r="I90" s="37"/>
       <x:c r="J90" s="37"/>
       <x:c r="K90" s="40"/>
-      <x:c r="L90" s="38"/>
-      <x:c r="M90" s="38"/>
-      <x:c r="N90" s="38"/>
+      <x:c r="L90" s="39"/>
+      <x:c r="M90" s="37"/>
+      <x:c r="N90" s="37"/>
+      <x:c r="O90" s="37"/>
+      <x:c r="P90" s="37"/>
+      <x:c r="Q90" s="38"/>
+      <x:c r="R90" s="38"/>
+      <x:c r="S90" s="38"/>
     </x:row>
     <x:row r="91" ht="24" customHeight="1">
       <x:c r="A91" s="37"/>
@@ -16099,9 +16569,14 @@
       <x:c r="I91" s="37"/>
       <x:c r="J91" s="37"/>
       <x:c r="K91" s="40"/>
-      <x:c r="L91" s="38"/>
-      <x:c r="M91" s="38"/>
-      <x:c r="N91" s="38"/>
+      <x:c r="L91" s="39"/>
+      <x:c r="M91" s="37"/>
+      <x:c r="N91" s="37"/>
+      <x:c r="O91" s="37"/>
+      <x:c r="P91" s="37"/>
+      <x:c r="Q91" s="38"/>
+      <x:c r="R91" s="38"/>
+      <x:c r="S91" s="38"/>
     </x:row>
     <x:row r="92" ht="24" customHeight="1">
       <x:c r="A92" s="37"/>
@@ -16115,9 +16590,14 @@
       <x:c r="I92" s="37"/>
       <x:c r="J92" s="37"/>
       <x:c r="K92" s="40"/>
-      <x:c r="L92" s="38"/>
-      <x:c r="M92" s="38"/>
-      <x:c r="N92" s="38"/>
+      <x:c r="L92" s="39"/>
+      <x:c r="M92" s="37"/>
+      <x:c r="N92" s="37"/>
+      <x:c r="O92" s="37"/>
+      <x:c r="P92" s="37"/>
+      <x:c r="Q92" s="38"/>
+      <x:c r="R92" s="38"/>
+      <x:c r="S92" s="38"/>
     </x:row>
     <x:row r="93" ht="24" customHeight="1">
       <x:c r="A93" s="37"/>
@@ -16131,9 +16611,14 @@
       <x:c r="I93" s="37"/>
       <x:c r="J93" s="37"/>
       <x:c r="K93" s="40"/>
-      <x:c r="L93" s="38"/>
-      <x:c r="M93" s="38"/>
-      <x:c r="N93" s="38"/>
+      <x:c r="L93" s="39"/>
+      <x:c r="M93" s="37"/>
+      <x:c r="N93" s="37"/>
+      <x:c r="O93" s="37"/>
+      <x:c r="P93" s="37"/>
+      <x:c r="Q93" s="38"/>
+      <x:c r="R93" s="38"/>
+      <x:c r="S93" s="38"/>
     </x:row>
     <x:row r="94" ht="24" customHeight="1">
       <x:c r="A94" s="37"/>
@@ -16147,9 +16632,14 @@
       <x:c r="I94" s="37"/>
       <x:c r="J94" s="37"/>
       <x:c r="K94" s="40"/>
-      <x:c r="L94" s="38"/>
-      <x:c r="M94" s="38"/>
-      <x:c r="N94" s="38"/>
+      <x:c r="L94" s="39"/>
+      <x:c r="M94" s="37"/>
+      <x:c r="N94" s="37"/>
+      <x:c r="O94" s="37"/>
+      <x:c r="P94" s="37"/>
+      <x:c r="Q94" s="38"/>
+      <x:c r="R94" s="38"/>
+      <x:c r="S94" s="38"/>
     </x:row>
     <x:row r="95" ht="24" customHeight="1">
       <x:c r="A95" s="37"/>
@@ -16163,9 +16653,14 @@
       <x:c r="I95" s="37"/>
       <x:c r="J95" s="37"/>
       <x:c r="K95" s="40"/>
-      <x:c r="L95" s="38"/>
-      <x:c r="M95" s="38"/>
-      <x:c r="N95" s="38"/>
+      <x:c r="L95" s="39"/>
+      <x:c r="M95" s="37"/>
+      <x:c r="N95" s="37"/>
+      <x:c r="O95" s="37"/>
+      <x:c r="P95" s="37"/>
+      <x:c r="Q95" s="38"/>
+      <x:c r="R95" s="38"/>
+      <x:c r="S95" s="38"/>
     </x:row>
     <x:row r="96" ht="24" customHeight="1">
       <x:c r="A96" s="37"/>
@@ -16179,9 +16674,14 @@
       <x:c r="I96" s="37"/>
       <x:c r="J96" s="37"/>
       <x:c r="K96" s="40"/>
-      <x:c r="L96" s="38"/>
-      <x:c r="M96" s="38"/>
-      <x:c r="N96" s="38"/>
+      <x:c r="L96" s="39"/>
+      <x:c r="M96" s="37"/>
+      <x:c r="N96" s="37"/>
+      <x:c r="O96" s="37"/>
+      <x:c r="P96" s="37"/>
+      <x:c r="Q96" s="38"/>
+      <x:c r="R96" s="38"/>
+      <x:c r="S96" s="38"/>
     </x:row>
     <x:row r="97" ht="24" customHeight="1">
       <x:c r="A97" s="37"/>
@@ -16195,9 +16695,14 @@
       <x:c r="I97" s="37"/>
       <x:c r="J97" s="37"/>
       <x:c r="K97" s="40"/>
-      <x:c r="L97" s="38"/>
-      <x:c r="M97" s="38"/>
-      <x:c r="N97" s="38"/>
+      <x:c r="L97" s="39"/>
+      <x:c r="M97" s="37"/>
+      <x:c r="N97" s="37"/>
+      <x:c r="O97" s="37"/>
+      <x:c r="P97" s="37"/>
+      <x:c r="Q97" s="38"/>
+      <x:c r="R97" s="38"/>
+      <x:c r="S97" s="38"/>
     </x:row>
     <x:row r="98" ht="24" customHeight="1">
       <x:c r="A98" s="37"/>
@@ -16211,9 +16716,14 @@
       <x:c r="I98" s="37"/>
       <x:c r="J98" s="37"/>
       <x:c r="K98" s="40"/>
-      <x:c r="L98" s="38"/>
-      <x:c r="M98" s="38"/>
-      <x:c r="N98" s="38"/>
+      <x:c r="L98" s="39"/>
+      <x:c r="M98" s="37"/>
+      <x:c r="N98" s="37"/>
+      <x:c r="O98" s="37"/>
+      <x:c r="P98" s="37"/>
+      <x:c r="Q98" s="38"/>
+      <x:c r="R98" s="38"/>
+      <x:c r="S98" s="38"/>
     </x:row>
     <x:row r="99" ht="24" customHeight="1">
       <x:c r="A99" s="37"/>
@@ -16227,9 +16737,14 @@
       <x:c r="I99" s="37"/>
       <x:c r="J99" s="37"/>
       <x:c r="K99" s="40"/>
-      <x:c r="L99" s="38"/>
-      <x:c r="M99" s="38"/>
-      <x:c r="N99" s="38"/>
+      <x:c r="L99" s="39"/>
+      <x:c r="M99" s="37"/>
+      <x:c r="N99" s="37"/>
+      <x:c r="O99" s="37"/>
+      <x:c r="P99" s="37"/>
+      <x:c r="Q99" s="38"/>
+      <x:c r="R99" s="38"/>
+      <x:c r="S99" s="38"/>
     </x:row>
     <x:row r="100" ht="24" customHeight="1">
       <x:c r="A100" s="37"/>
@@ -16243,9 +16758,14 @@
       <x:c r="I100" s="37"/>
       <x:c r="J100" s="37"/>
       <x:c r="K100" s="40"/>
-      <x:c r="L100" s="38"/>
-      <x:c r="M100" s="38"/>
-      <x:c r="N100" s="38"/>
+      <x:c r="L100" s="39"/>
+      <x:c r="M100" s="37"/>
+      <x:c r="N100" s="37"/>
+      <x:c r="O100" s="37"/>
+      <x:c r="P100" s="37"/>
+      <x:c r="Q100" s="38"/>
+      <x:c r="R100" s="38"/>
+      <x:c r="S100" s="38"/>
     </x:row>
     <x:row r="101" ht="24" customHeight="1">
       <x:c r="A101" s="37"/>
@@ -16259,9 +16779,14 @@
       <x:c r="I101" s="37"/>
       <x:c r="J101" s="37"/>
       <x:c r="K101" s="40"/>
-      <x:c r="L101" s="38"/>
-      <x:c r="M101" s="38"/>
-      <x:c r="N101" s="38"/>
+      <x:c r="L101" s="39"/>
+      <x:c r="M101" s="37"/>
+      <x:c r="N101" s="37"/>
+      <x:c r="O101" s="37"/>
+      <x:c r="P101" s="37"/>
+      <x:c r="Q101" s="38"/>
+      <x:c r="R101" s="38"/>
+      <x:c r="S101" s="38"/>
     </x:row>
     <x:row r="102" ht="24" customHeight="1">
       <x:c r="A102" s="37"/>
@@ -16275,9 +16800,14 @@
       <x:c r="I102" s="37"/>
       <x:c r="J102" s="37"/>
       <x:c r="K102" s="40"/>
-      <x:c r="L102" s="38"/>
-      <x:c r="M102" s="38"/>
-      <x:c r="N102" s="38"/>
+      <x:c r="L102" s="39"/>
+      <x:c r="M102" s="37"/>
+      <x:c r="N102" s="37"/>
+      <x:c r="O102" s="37"/>
+      <x:c r="P102" s="37"/>
+      <x:c r="Q102" s="38"/>
+      <x:c r="R102" s="38"/>
+      <x:c r="S102" s="38"/>
     </x:row>
     <x:row r="103" ht="24" customHeight="1">
       <x:c r="A103" s="37"/>
@@ -16291,9 +16821,14 @@
       <x:c r="I103" s="37"/>
       <x:c r="J103" s="37"/>
       <x:c r="K103" s="40"/>
-      <x:c r="L103" s="38"/>
-      <x:c r="M103" s="38"/>
-      <x:c r="N103" s="38"/>
+      <x:c r="L103" s="39"/>
+      <x:c r="M103" s="37"/>
+      <x:c r="N103" s="37"/>
+      <x:c r="O103" s="37"/>
+      <x:c r="P103" s="37"/>
+      <x:c r="Q103" s="38"/>
+      <x:c r="R103" s="38"/>
+      <x:c r="S103" s="38"/>
     </x:row>
     <x:row r="104" ht="24" customHeight="1">
       <x:c r="A104" s="37"/>
@@ -16307,19 +16842,24 @@
       <x:c r="I104" s="37"/>
       <x:c r="J104" s="37"/>
       <x:c r="K104" s="40"/>
-      <x:c r="L104" s="38"/>
-      <x:c r="M104" s="38"/>
-      <x:c r="N104" s="38"/>
+      <x:c r="L104" s="39"/>
+      <x:c r="M104" s="37"/>
+      <x:c r="N104" s="37"/>
+      <x:c r="O104" s="37"/>
+      <x:c r="P104" s="37"/>
+      <x:c r="Q104" s="38"/>
+      <x:c r="R104" s="38"/>
+      <x:c r="S104" s="38"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:N1"/>
-    <x:mergeCell ref="A2:N2"/>
-    <x:mergeCell ref="A3:N3"/>
+    <x:mergeCell ref="A1:S1"/>
+    <x:mergeCell ref="A2:S2"/>
+    <x:mergeCell ref="A3:S3"/>
   </x:mergeCells>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="B5:B104">
-      <x:formula1>"overview,devotional,instruction,itinerary,resource,update"</x:formula1>
+      <x:formula1>"overview,devotional,instruction,itinerary,travel,resource,update"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="I5:I104">
       <x:formula1>"public,travelers,admin"</x:formula1>
@@ -16330,7 +16870,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88884bd895c44b80"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R589a0a72bd5f4a50"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17968,7 +18508,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc748eba30e24291"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08c9b4d556484065"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20679,7 +21219,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5219ab4a30e94e80"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref54630269814a99"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21883,7 +22423,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf63b56ce6fa742b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e21d1a828cd48d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>